<commit_message>
cal metrics for gemma4 with temperature
</commit_message>
<xml_diff>
--- a/src/results/llm/temperature_testing_01/results_for_presentation_temperature_testing.xlsx
+++ b/src/results/llm/temperature_testing_01/results_for_presentation_temperature_testing.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\Using-LLM-for-automated-feedback-generation-on-a-bachelor-thesis\src\results\llm\temperature_testing_01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D85653A2-6D0A-4455-8CA8-A6616FDE22D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDE75E1D-6BA2-4394-A070-8FA02FE29F02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="GPT-OSS-20b" sheetId="1" r:id="rId1"/>
+    <sheet name="gemma4-26b-q4" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="12">
   <si>
     <t>temperatūra</t>
   </si>
@@ -123,22 +124,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -423,73 +429,73 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="20.140625" style="10" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" style="10" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" style="10" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" style="10" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" style="10" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" style="8" customWidth="1"/>
+    <col min="3" max="3" width="20.85546875" style="8" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" style="8" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="8" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" style="8" customWidth="1"/>
     <col min="7" max="7" width="9.140625" style="1"/>
     <col min="8" max="8" width="15.85546875" style="4" customWidth="1"/>
-    <col min="9" max="9" width="18.5703125" style="10" customWidth="1"/>
-    <col min="10" max="10" width="19" style="10" customWidth="1"/>
-    <col min="11" max="11" width="13" style="10" customWidth="1"/>
-    <col min="12" max="12" width="12.140625" style="10" customWidth="1"/>
-    <col min="13" max="13" width="13.28515625" style="10" customWidth="1"/>
+    <col min="9" max="9" width="18.5703125" style="8" customWidth="1"/>
+    <col min="10" max="10" width="19" style="8" customWidth="1"/>
+    <col min="11" max="11" width="13" style="8" customWidth="1"/>
+    <col min="12" max="12" width="12.140625" style="8" customWidth="1"/>
+    <col min="13" max="13" width="13.28515625" style="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="H1" s="7" t="s">
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="H1" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="8" t="s">
+      <c r="B2" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="6" t="s">
         <v>5</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="I2" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="J2" s="8" t="s">
+      <c r="I2" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="J2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="K2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="L2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="M2" s="6" t="s">
         <v>5</v>
       </c>
     </row>
@@ -497,37 +503,37 @@
       <c r="A3" s="3">
         <v>0</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="11">
         <v>0.90079784918781403</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="11">
         <v>0.85302197802197699</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="11">
         <v>0.87624973584661003</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="11">
         <v>0.85168636941259801</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="11">
         <v>0.70368404512316896</v>
       </c>
       <c r="H3" s="3">
         <v>0</v>
       </c>
-      <c r="I3" s="9">
+      <c r="I3" s="11">
         <v>2.9136181726262299E-3</v>
       </c>
-      <c r="J3" s="9">
+      <c r="J3" s="11">
         <v>3.9334673250758997E-3</v>
       </c>
-      <c r="K3" s="9">
+      <c r="K3" s="11">
         <v>2.0200156267348801E-3</v>
       </c>
-      <c r="L3" s="9">
+      <c r="L3" s="11">
         <v>2.24649152789945E-3</v>
       </c>
-      <c r="M3" s="9">
+      <c r="M3" s="11">
         <v>4.4760786228040302E-3</v>
       </c>
     </row>
@@ -535,37 +541,37 @@
       <c r="A4" s="3">
         <v>0.5</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="11">
         <v>0.90452780922405995</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="11">
         <v>0.83131868131868103</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="11">
         <v>0.86634686155859597</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="11">
         <v>0.84297889063682097</v>
       </c>
-      <c r="F4" s="9">
+      <c r="F4" s="11">
         <v>0.68672719365495505</v>
       </c>
       <c r="H4" s="3">
         <v>0.5</v>
       </c>
-      <c r="I4" s="9">
+      <c r="I4" s="11">
         <v>6.5122422347781801E-3</v>
       </c>
-      <c r="J4" s="9">
+      <c r="J4" s="11">
         <v>9.7479093402253695E-3</v>
       </c>
-      <c r="K4" s="9">
+      <c r="K4" s="11">
         <v>6.6599573790513504E-3</v>
       </c>
-      <c r="L4" s="9">
+      <c r="L4" s="11">
         <v>7.2637750227528301E-3</v>
       </c>
-      <c r="M4" s="9">
+      <c r="M4" s="11">
         <v>1.44101747321142E-2</v>
       </c>
     </row>
@@ -573,93 +579,93 @@
       <c r="A5" s="3">
         <v>1</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="11">
         <v>0.90448335311697203</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="11">
         <v>0.81414835164835098</v>
       </c>
-      <c r="D5" s="9">
+      <c r="D5" s="11">
         <v>0.85691405597203496</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="11">
         <v>0.83411282542487297</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="11">
         <v>0.66944772824958798</v>
       </c>
       <c r="H5" s="3">
         <v>1</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="11">
         <v>4.9133078389275798E-3</v>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="11">
         <v>9.3578139177203697E-3</v>
       </c>
-      <c r="K5" s="9">
+      <c r="K5" s="11">
         <v>6.1590328433094796E-3</v>
       </c>
-      <c r="L5" s="9">
+      <c r="L5" s="11">
         <v>6.3865113196029701E-3</v>
       </c>
-      <c r="M5" s="9">
+      <c r="M5" s="11">
         <v>1.2577494328024E-2</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="H8" s="7" t="s">
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="H8" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="I8" s="7"/>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C9" s="8" t="s">
+      <c r="B9" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="6" t="s">
         <v>5</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="I9" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="J9" s="8" t="s">
+      <c r="I9" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="J9" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="K9" s="8" t="s">
+      <c r="K9" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="L9" s="8" t="s">
+      <c r="L9" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="M9" s="8" t="s">
+      <c r="M9" s="6" t="s">
         <v>5</v>
       </c>
     </row>
@@ -667,37 +673,37 @@
       <c r="A10" s="3">
         <v>0</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="11">
         <v>0.71439661370665997</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="11">
         <v>0.86403508771929804</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="11">
         <v>0.78211444101669403</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="11">
         <v>0.77405126857954498</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="11">
         <v>0.55242888231745602</v>
       </c>
       <c r="H10" s="3">
         <v>0</v>
       </c>
-      <c r="I10" s="9">
+      <c r="I10" s="11">
         <v>3.6598128491763401E-3</v>
       </c>
-      <c r="J10" s="9">
+      <c r="J10" s="11">
         <v>6.0392682379152799E-3</v>
       </c>
-      <c r="K10" s="9">
+      <c r="K10" s="11">
         <v>3.9647617982254803E-3</v>
       </c>
-      <c r="L10" s="9">
+      <c r="L10" s="11">
         <v>3.9452728520661898E-3</v>
       </c>
-      <c r="M10" s="9">
+      <c r="M10" s="11">
         <v>7.8525171554414096E-3</v>
       </c>
     </row>
@@ -705,37 +711,37 @@
       <c r="A11" s="3">
         <v>0.5</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="11">
         <v>0.724454828535535</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="11">
         <v>0.85035087719298197</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="11">
         <v>0.78234118122740604</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="11">
         <v>0.77811664907407097</v>
       </c>
-      <c r="F11" s="9">
+      <c r="F11" s="11">
         <v>0.55918510422869205</v>
       </c>
       <c r="H11" s="3">
         <v>0.5</v>
       </c>
-      <c r="I11" s="9">
+      <c r="I11" s="11">
         <v>8.6293253318535205E-3</v>
       </c>
-      <c r="J11" s="9">
+      <c r="J11" s="11">
         <v>1.07017543859649E-2</v>
       </c>
-      <c r="K11" s="9">
+      <c r="K11" s="11">
         <v>8.27661678061406E-3</v>
       </c>
-      <c r="L11" s="9">
+      <c r="L11" s="11">
         <v>8.5592441537415999E-3</v>
       </c>
-      <c r="M11" s="9">
+      <c r="M11" s="11">
         <v>1.6930568497639301E-2</v>
       </c>
     </row>
@@ -743,93 +749,93 @@
       <c r="A12" s="3">
         <v>1</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="11">
         <v>0.72670720301903502</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="11">
         <v>0.83543859649122798</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="11">
         <v>0.77726358537395801</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="11">
         <v>0.77555425295750502</v>
       </c>
-      <c r="F12" s="9">
+      <c r="F12" s="11">
         <v>0.55332109327637202</v>
       </c>
       <c r="H12" s="3">
         <v>1</v>
       </c>
-      <c r="I12" s="9">
+      <c r="I12" s="11">
         <v>6.0861439214959998E-3</v>
       </c>
-      <c r="J12" s="9">
+      <c r="J12" s="11">
         <v>1.03731547362066E-2</v>
       </c>
-      <c r="K12" s="9">
+      <c r="K12" s="11">
         <v>6.7988854894443897E-3</v>
       </c>
-      <c r="L12" s="9">
+      <c r="L12" s="11">
         <v>6.4846177674893002E-3</v>
       </c>
-      <c r="M12" s="9">
+      <c r="M12" s="11">
         <v>1.2979957128324201E-2</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="H15" s="7" t="s">
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="H15" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I15" s="7"/>
-      <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
-      <c r="L15" s="7"/>
-      <c r="M15" s="7"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C16" s="8" t="s">
+      <c r="B16" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="6" t="s">
         <v>5</v>
       </c>
       <c r="H16" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="I16" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="J16" s="8" t="s">
+      <c r="I16" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="J16" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="K16" s="8" t="s">
+      <c r="K16" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="L16" s="8" t="s">
+      <c r="L16" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="M16" s="8" t="s">
+      <c r="M16" s="6" t="s">
         <v>5</v>
       </c>
     </row>
@@ -837,37 +843,37 @@
       <c r="A17" s="3">
         <v>0</v>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="11">
         <v>0.913409718540237</v>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="11">
         <v>0.78909774436090196</v>
       </c>
-      <c r="D17" s="9">
+      <c r="D17" s="11">
         <v>0.84670617757195399</v>
       </c>
-      <c r="E17" s="9">
+      <c r="E17" s="11">
         <v>0.80267028107066396</v>
       </c>
-      <c r="F17" s="9">
+      <c r="F17" s="11">
         <v>0.60863315572362298</v>
       </c>
       <c r="H17" s="3">
         <v>0</v>
       </c>
-      <c r="I17" s="9">
+      <c r="I17" s="11">
         <v>2.6542969022385799E-3</v>
       </c>
-      <c r="J17" s="9">
+      <c r="J17" s="11">
         <v>4.7898533467710296E-3</v>
       </c>
-      <c r="K17" s="9">
+      <c r="K17" s="11">
         <v>3.04257830547882E-3</v>
       </c>
-      <c r="L17" s="9">
+      <c r="L17" s="11">
         <v>3.3639788023401098E-3</v>
       </c>
-      <c r="M17" s="9">
+      <c r="M17" s="11">
         <v>6.5463403956715401E-3</v>
       </c>
     </row>
@@ -875,37 +881,37 @@
       <c r="A18" s="3">
         <v>0.5</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="11">
         <v>0.91182264880127795</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="11">
         <v>0.76453634085212996</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="11">
         <v>0.83167800119479796</v>
       </c>
-      <c r="E18" s="9">
+      <c r="E18" s="11">
         <v>0.78791842037030702</v>
       </c>
-      <c r="F18" s="9">
+      <c r="F18" s="11">
         <v>0.58078964796676702</v>
       </c>
       <c r="H18" s="3">
         <v>0.5</v>
       </c>
-      <c r="I18" s="9">
+      <c r="I18" s="11">
         <v>2.8120418560879002E-3</v>
       </c>
-      <c r="J18" s="9">
+      <c r="J18" s="11">
         <v>9.6328346070063305E-3</v>
       </c>
-      <c r="K18" s="9">
+      <c r="K18" s="11">
         <v>6.0731585006510297E-3</v>
       </c>
-      <c r="L18" s="9">
+      <c r="L18" s="11">
         <v>6.0614447631849398E-3</v>
       </c>
-      <c r="M18" s="9">
+      <c r="M18" s="11">
         <v>1.147090341247E-2</v>
       </c>
     </row>
@@ -913,37 +919,37 @@
       <c r="A19" s="3">
         <v>1</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="11">
         <v>0.91243209757064603</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="11">
         <v>0.74924812030075105</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="11">
         <v>0.82280093560758305</v>
       </c>
-      <c r="E19" s="9">
+      <c r="E19" s="11">
         <v>0.77985326663184595</v>
       </c>
-      <c r="F19" s="9">
+      <c r="F19" s="11">
         <v>0.56594201035421798</v>
       </c>
       <c r="H19" s="3">
         <v>1</v>
       </c>
-      <c r="I19" s="9">
+      <c r="I19" s="11">
         <v>4.4385669546764001E-3</v>
       </c>
-      <c r="J19" s="9">
+      <c r="J19" s="11">
         <v>7.4019746494347598E-3</v>
       </c>
-      <c r="K19" s="9">
+      <c r="K19" s="11">
         <v>4.6689934132352496E-3</v>
       </c>
-      <c r="L19" s="9">
+      <c r="L19" s="11">
         <v>4.8314818804129798E-3</v>
       </c>
-      <c r="M19" s="9">
+      <c r="M19" s="11">
         <v>9.2523659633384804E-3</v>
       </c>
     </row>
@@ -958,4 +964,577 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E0FD20B-D6B3-444D-8CDB-F1C6BAEC8830}">
+  <dimension ref="A1:M19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="21" style="8" customWidth="1"/>
+    <col min="3" max="3" width="23" style="8" customWidth="1"/>
+    <col min="4" max="4" width="15.42578125" style="8" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" style="8" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" style="8" customWidth="1"/>
+    <col min="8" max="8" width="16" style="8" customWidth="1"/>
+    <col min="9" max="9" width="23" style="8" customWidth="1"/>
+    <col min="10" max="10" width="18.42578125" style="8" customWidth="1"/>
+    <col min="11" max="11" width="17.28515625" style="8" customWidth="1"/>
+    <col min="12" max="12" width="17" style="8" customWidth="1"/>
+    <col min="13" max="13" width="15.5703125" style="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="1"/>
+      <c r="H2" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>0</v>
+      </c>
+      <c r="B3" s="8">
+        <v>0.86658195679796601</v>
+      </c>
+      <c r="C3" s="8">
+        <v>0.93681318681318604</v>
+      </c>
+      <c r="D3" s="8">
+        <v>0.90033003300329995</v>
+      </c>
+      <c r="E3" s="8">
+        <v>0.86783131966413596</v>
+      </c>
+      <c r="F3" s="8">
+        <v>0.73632332330032302</v>
+      </c>
+      <c r="G3" s="1"/>
+      <c r="H3" s="7">
+        <v>0</v>
+      </c>
+      <c r="I3" s="12">
+        <v>0</v>
+      </c>
+      <c r="J3" s="8">
+        <v>0</v>
+      </c>
+      <c r="K3" s="8">
+        <v>0</v>
+      </c>
+      <c r="L3" s="8">
+        <v>0</v>
+      </c>
+      <c r="M3" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="B4" s="8">
+        <v>0.86470422231483601</v>
+      </c>
+      <c r="C4" s="8">
+        <v>0.94464285714285701</v>
+      </c>
+      <c r="D4" s="8">
+        <v>0.90290345278527495</v>
+      </c>
+      <c r="E4" s="8">
+        <v>0.87007647968240898</v>
+      </c>
+      <c r="F4" s="8">
+        <v>0.74100120292315597</v>
+      </c>
+      <c r="G4" s="1"/>
+      <c r="H4" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="I4" s="8">
+        <v>1.5825144691276401E-3</v>
+      </c>
+      <c r="J4" s="8">
+        <v>4.6399301522127602E-3</v>
+      </c>
+      <c r="K4" s="8">
+        <v>2.6523160355263801E-3</v>
+      </c>
+      <c r="L4" s="8">
+        <v>3.1729453716925699E-3</v>
+      </c>
+      <c r="M4" s="8">
+        <v>6.3891111178268596E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8">
+        <v>0.86398282763146395</v>
+      </c>
+      <c r="C5" s="8">
+        <v>0.93804945054944999</v>
+      </c>
+      <c r="D5" s="8">
+        <v>0.89948390781018805</v>
+      </c>
+      <c r="E5" s="8">
+        <v>0.86624316615166796</v>
+      </c>
+      <c r="F5" s="8">
+        <v>0.73323581734427201</v>
+      </c>
+      <c r="G5" s="1"/>
+      <c r="H5" s="7">
+        <v>1</v>
+      </c>
+      <c r="I5" s="8">
+        <v>2.7816543924288699E-3</v>
+      </c>
+      <c r="J5" s="8">
+        <v>8.3203668796196593E-3</v>
+      </c>
+      <c r="K5" s="8">
+        <v>5.08266169141344E-3</v>
+      </c>
+      <c r="L5" s="8">
+        <v>6.0980346746056799E-3</v>
+      </c>
+      <c r="M5" s="8">
+        <v>1.2269072714577599E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="4"/>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="4"/>
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I8" s="13"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="13"/>
+      <c r="L8" s="13"/>
+      <c r="M8" s="13"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G9" s="1"/>
+      <c r="H9" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="M9" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
+        <v>0</v>
+      </c>
+      <c r="B10" s="8">
+        <v>0.677255400254129</v>
+      </c>
+      <c r="C10" s="8">
+        <v>0.93508771929824497</v>
+      </c>
+      <c r="D10" s="8">
+        <v>0.78555637435519499</v>
+      </c>
+      <c r="E10" s="8">
+        <v>0.75742934996829503</v>
+      </c>
+      <c r="F10" s="8">
+        <v>0.530029272231755</v>
+      </c>
+      <c r="G10" s="1"/>
+      <c r="H10" s="7">
+        <v>0</v>
+      </c>
+      <c r="I10" s="8">
+        <v>0</v>
+      </c>
+      <c r="J10" s="8">
+        <v>0</v>
+      </c>
+      <c r="K10" s="8">
+        <v>0</v>
+      </c>
+      <c r="L10" s="8">
+        <v>0</v>
+      </c>
+      <c r="M10" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="B11" s="8">
+        <v>0.678108385709152</v>
+      </c>
+      <c r="C11" s="8">
+        <v>0.94614035087719295</v>
+      </c>
+      <c r="D11" s="8">
+        <v>0.79000559950443905</v>
+      </c>
+      <c r="E11" s="8">
+        <v>0.76061708189307897</v>
+      </c>
+      <c r="F11" s="8">
+        <v>0.53736061265073598</v>
+      </c>
+      <c r="G11" s="1"/>
+      <c r="H11" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="I11" s="8">
+        <v>3.2766920511978601E-3</v>
+      </c>
+      <c r="J11" s="8">
+        <v>6.2299231244086397E-3</v>
+      </c>
+      <c r="K11" s="8">
+        <v>4.1202598423994699E-3</v>
+      </c>
+      <c r="L11" s="8">
+        <v>4.4556769780229096E-3</v>
+      </c>
+      <c r="M11" s="8">
+        <v>8.7360066675477906E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>1</v>
+      </c>
+      <c r="B12" s="8">
+        <v>0.67850898277712401</v>
+      </c>
+      <c r="C12" s="8">
+        <v>0.94087719298245598</v>
+      </c>
+      <c r="D12" s="8">
+        <v>0.78843038376132402</v>
+      </c>
+      <c r="E12" s="8">
+        <v>0.75993558816800999</v>
+      </c>
+      <c r="F12" s="8">
+        <v>0.53535335397119299</v>
+      </c>
+      <c r="G12" s="1"/>
+      <c r="H12" s="7">
+        <v>1</v>
+      </c>
+      <c r="I12" s="8">
+        <v>2.7393041358206899E-3</v>
+      </c>
+      <c r="J12" s="8">
+        <v>8.7032398279385508E-3</v>
+      </c>
+      <c r="K12" s="8">
+        <v>4.6234739381984099E-3</v>
+      </c>
+      <c r="L12" s="8">
+        <v>4.3780834165333404E-3</v>
+      </c>
+      <c r="M12" s="8">
+        <v>8.9825721331164999E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" s="4"/>
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" s="4"/>
+      <c r="G14" s="1"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="I15" s="13"/>
+      <c r="J15" s="13"/>
+      <c r="K15" s="13"/>
+      <c r="L15" s="13"/>
+      <c r="M15" s="13"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G16" s="1"/>
+      <c r="H16" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="M16" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
+        <v>0</v>
+      </c>
+      <c r="B17" s="8">
+        <v>0.89199491740787795</v>
+      </c>
+      <c r="C17" s="8">
+        <v>0.87969924812029998</v>
+      </c>
+      <c r="D17" s="8">
+        <v>0.88580441640378504</v>
+      </c>
+      <c r="E17" s="8">
+        <v>0.83605451044510404</v>
+      </c>
+      <c r="F17" s="8">
+        <v>0.67213857126683996</v>
+      </c>
+      <c r="G17" s="1"/>
+      <c r="H17" s="7">
+        <v>0</v>
+      </c>
+      <c r="I17" s="8">
+        <v>0</v>
+      </c>
+      <c r="J17" s="8">
+        <v>0</v>
+      </c>
+      <c r="K17" s="8">
+        <v>0</v>
+      </c>
+      <c r="L17" s="8">
+        <v>0</v>
+      </c>
+      <c r="M17" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A18" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="B18" s="8">
+        <v>0.89111061145925796</v>
+      </c>
+      <c r="C18" s="8">
+        <v>0.88809523809523805</v>
+      </c>
+      <c r="D18" s="8">
+        <v>0.88959622419697404</v>
+      </c>
+      <c r="E18" s="8">
+        <v>0.83993788616379295</v>
+      </c>
+      <c r="F18" s="8">
+        <v>0.67988043932810005</v>
+      </c>
+      <c r="G18" s="1"/>
+      <c r="H18" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="I18" s="8">
+        <v>2.3394410523621101E-3</v>
+      </c>
+      <c r="J18" s="8">
+        <v>4.4145150260171797E-3</v>
+      </c>
+      <c r="K18" s="8">
+        <v>2.9750369323296002E-3</v>
+      </c>
+      <c r="L18" s="8">
+        <v>3.9247325753674596E-3</v>
+      </c>
+      <c r="M18" s="8">
+        <v>7.8450627154047492E-3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" s="3">
+        <v>1</v>
+      </c>
+      <c r="B19" s="8">
+        <v>0.89068807962548202</v>
+      </c>
+      <c r="C19" s="8">
+        <v>0.88220551378446099</v>
+      </c>
+      <c r="D19" s="8">
+        <v>0.88641653581075097</v>
+      </c>
+      <c r="E19" s="8">
+        <v>0.83629689588767397</v>
+      </c>
+      <c r="F19" s="8">
+        <v>0.672615121309315</v>
+      </c>
+      <c r="G19" s="1"/>
+      <c r="H19" s="7">
+        <v>1</v>
+      </c>
+      <c r="I19" s="8">
+        <v>1.75585465191171E-3</v>
+      </c>
+      <c r="J19" s="8">
+        <v>6.19001956653056E-3</v>
+      </c>
+      <c r="K19" s="8">
+        <v>3.4855699905592201E-3</v>
+      </c>
+      <c r="L19" s="8">
+        <v>4.1677879017123299E-3</v>
+      </c>
+      <c r="M19" s="8">
+        <v>8.3177852835428102E-3</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="H1:M1"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="H8:M8"/>
+    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="H15:M15"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>